<commit_message>
Adding Cucumber and Some uncommited files
</commit_message>
<xml_diff>
--- a/src/main/resources/datapool/TestData.xlsx
+++ b/src/main/resources/datapool/TestData.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20378"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\RSPL_Selenium\rspl_qa_training_certification_r-d\src\main\resources\datapool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalpesh.deore\eclipse-workspace\rspl_Automation\rspl_qa_training_certification_r-d\src\main\resources\datapool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A95B78A8-8FE8-4579-A2D5-FDFAA1006D91}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC5DC12-9CA0-4584-BFD9-9841F0F0B48F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" activeTab="1" xr2:uid="{E8580097-6381-41A7-A50E-8A6FA3C5DEEE}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{E8580097-6381-41A7-A50E-8A6FA3C5DEEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet_User" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet_SearchModel" sheetId="3" r:id="rId3"/>
+    <sheet name="testdata" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>REPORT_FILENAME</t>
   </si>
@@ -102,6 +103,12 @@
   </si>
   <si>
     <t>E-Commerce</t>
+  </si>
+  <si>
+    <t>Expected Oppo ID</t>
+  </si>
+  <si>
+    <t>AI Model Deployment</t>
   </si>
 </sst>
 </file>
@@ -606,4 +613,28 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23E782C7-3B76-4AA4-9126-AF5AA81CA653}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>